<commit_message>
Close patch-coverage gaps and fix add-row context drop (#175)
Cover the documentRef extraction helpers (empty/list referenceDocuments,
absent referenceDocumentId, every pageRefs shape), the JSON inline+
documentRef mix with an empty-refId skip, and the XLSX add-row branch
(documentRef method with no AnalysisMethodCodeTemplate sheet row).

Fix a latent bug surfaced by that coverage: AnalysisMethods.R filters
templates on context %in% c('R','R (siera)','siera'), so a resolved
method whose row carried no context (the XLSX add-row branch, or a JSON
documentRef method that omits codeTemplate.context) was silently dropped.
The resolver now returns a context (manifest method's, else manifest-
level, else 'R (siera)') and both metadata paths use it. The shipped
exampleARS_5_documentref.xlsx now exercises both the update and add-row
branches.
</commit_message>
<xml_diff>
--- a/inst/extdata/exampleARS_5_documentref.xlsx
+++ b/inst/extdata/exampleARS_5_documentref.xlsx
@@ -1032,70 +1032,70 @@
     <t xml:space="preserve">Code</t>
   </si>
   <si>
+    <t xml:space="preserve">parameter_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parameter_description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parameter_label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parameter_valueSource</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parameter_value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RefDoc_siera_methods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">siera example method manifest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exampleARS_methods.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">referenceType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refDocumentId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pageRef_refType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pageRef_label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pageRef_pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ExternalCode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NamedDestination</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mth_02</t>
   </si>
   <si>
     <t xml:space="preserve">Mth_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parameter_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parameter_description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parameter_label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parameter_valueSource</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parameter_value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">location</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RefDoc_siera_methods</t>
-  </si>
-  <si>
-    <t xml:space="preserve">siera example method manifest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">exampleARS_methods.json</t>
-  </si>
-  <si>
-    <t xml:space="preserve">referenceType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">refDocumentId</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pageRef_refType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pageRef_label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pageRef_pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExternalCode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NamedDestination</t>
   </si>
 </sst>
 </file>
@@ -2693,32 +2693,32 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>307</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -3179,30 +3179,6 @@
       </c>
       <c r="D2"/>
     </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>298</v>
-      </c>
-      <c r="B3" t="s">
-        <v>296</v>
-      </c>
-      <c r="C3" t="s">
-        <v>297</v>
-      </c>
-      <c r="D3"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>299</v>
-      </c>
-      <c r="B4" t="s">
-        <v>296</v>
-      </c>
-      <c r="C4" t="s">
-        <v>297</v>
-      </c>
-      <c r="D4"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -3219,19 +3195,19 @@
         <v>291</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>302</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>304</v>
       </c>
     </row>
   </sheetData>
@@ -3250,19 +3226,19 @@
         <v>291</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="2">
@@ -3270,13 +3246,13 @@
         <v>295</v>
       </c>
       <c r="B2" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C2" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="E2" t="s">
         <v>295</v>
@@ -3287,42 +3263,42 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>298</v>
+        <v>318</v>
       </c>
       <c r="B3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C3" t="s">
+        <v>308</v>
+      </c>
+      <c r="D3" t="s">
+        <v>317</v>
+      </c>
+      <c r="E3" t="s">
         <v>318</v>
       </c>
-      <c r="C3" t="s">
-        <v>310</v>
-      </c>
-      <c r="D3" t="s">
-        <v>319</v>
-      </c>
-      <c r="E3" t="s">
-        <v>298</v>
-      </c>
       <c r="F3" t="s">
-        <v>298</v>
+        <v>318</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>299</v>
+        <v>319</v>
       </c>
       <c r="B4" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C4" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D4" t="s">
+        <v>317</v>
+      </c>
+      <c r="E4" t="s">
         <v>319</v>
       </c>
-      <c r="E4" t="s">
-        <v>299</v>
-      </c>
       <c r="F4" t="s">
-        <v>299</v>
+        <v>319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>